<commit_message>
Address Codex review round 1: crawler cache scoping, unresolved-size handling, Excel table range
- crawl_release.py: keep manifest rows whose size lookup failed (preserve previous
  size, report them) instead of silently dropping them; key the listing cache by
  ROOT and restrict the shared size cache to the requested scope so a subtree run
  cannot poison a release-wide run (and vice versa).
- build_xlsx.py: resize MasterCatalogTable (and autofilter) to the regenerated
  row count so new datasets are inside the Excel table.
- GIAB_HG_Catalog.xlsx: table range A4:AY338 (was A4:AY336).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAB_HG_Catalog.xlsx
+++ b/GIAB_HG_Catalog.xlsx
@@ -542,7 +542,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterCatalogTable" displayName="MasterCatalogTable" ref="A4:AY336" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterCatalogTable" displayName="MasterCatalogTable" ref="A4:AY338" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="51">
     <tableColumn id="1" name="sample"/>
     <tableColumn id="2" name="category"/>
@@ -1494,7 +1494,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -3231,7 +3230,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -3316,8 +3314,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -3457,7 +3453,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="28" t="inlineStr">
         <is>
@@ -3513,7 +3508,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="45" t="inlineStr">
         <is>

</xml_diff>